<commit_message>
Fix supplementary tables to 104-gene analysis set; sync figures; remove orphan sparsity figure
- tables/TableS1-5.xlsx: corrected gene counts (104/73/104/30/11), added Legend sheets, renamed data sheets to S1-S5
- tables/TableS1-3.csv & data/processed/covariate_matrix.csv: removed 10 low-confidence non-candidate genes (Unused<2.0) erroneously re-included; now 104 genes, consistent with downstream analysis log
- tables/TableS3-5_legend.txt: fixed S-number offset (S4/S5/S6 -> S3/S4/S5)
- figures/ & supplementary/: synced Figure 1-9 and Figure S1-8
- supplementary/: removed orphan FigureS_sparsity_robustness (not cited in manuscript/SI)
</commit_message>
<xml_diff>
--- a/tables/TableS1.xlsx
+++ b/tables/TableS1.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS1_gene_list" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:J105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -864,7 +865,6 @@
       <c r="I11" t="n">
         <v>48.1</v>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -902,7 +902,6 @@
       <c r="I12" t="n">
         <v>46.3</v>
       </c>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1300,7 +1299,6 @@
       <c r="I22" t="n">
         <v>46</v>
       </c>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1778,7 +1776,6 @@
       <c r="I34" t="n">
         <v>42.1</v>
       </c>
-      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1816,7 +1813,6 @@
       <c r="I35" t="n">
         <v>41.8</v>
       </c>
-      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1894,7 +1890,6 @@
       <c r="I37" t="n">
         <v>67.40000000000001</v>
       </c>
-      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2012,7 +2007,6 @@
       <c r="I40" t="n">
         <v>46.4</v>
       </c>
-      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2130,7 +2124,6 @@
       <c r="I43" t="n">
         <v>48.9</v>
       </c>
-      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2175,7 +2168,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>H2AJ</t>
+          <t>H2BC13</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2194,26 +2187,25 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1.74</v>
+        <v>9.82</v>
       </c>
       <c r="F45" t="n">
-        <v>20.9299996495247</v>
+        <v>42.059999704361</v>
       </c>
       <c r="G45" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H45" t="n">
-        <v>4441</v>
+        <v>5714</v>
       </c>
       <c r="I45" t="n">
-        <v>51</v>
-      </c>
-      <c r="J45" t="inlineStr"/>
+        <v>52.1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>H2BC13</t>
+          <t>HMGA1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2232,26 +2224,25 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>9.82</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
-        <v>42.059999704361</v>
+        <v>23.3600005507469</v>
       </c>
       <c r="G46" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H46" t="n">
-        <v>5714</v>
+        <v>28395</v>
       </c>
       <c r="I46" t="n">
-        <v>52.1</v>
-      </c>
-      <c r="J46" t="inlineStr"/>
+        <v>42.1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>H3-7</t>
+          <t>HNRNPK</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2270,26 +2261,25 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1.31</v>
+        <v>4.41</v>
       </c>
       <c r="F47" t="n">
-        <v>24.2599993944168</v>
+        <v>11.2300001084805</v>
       </c>
       <c r="G47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H47" t="n">
-        <v>19412</v>
+        <v>10786</v>
       </c>
       <c r="I47" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="J47" t="inlineStr"/>
+        <v>40.2</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>HMGA1</t>
+          <t>HNRNPU</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2308,26 +2298,25 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
-        <v>23.3600005507469</v>
+        <v>7.15200006961823</v>
       </c>
       <c r="G48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H48" t="n">
-        <v>28395</v>
+        <v>26403</v>
       </c>
       <c r="I48" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="J48" t="inlineStr"/>
+        <v>43.8</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HNRNPK</t>
+          <t>HSPB1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2342,30 +2331,32 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>4.41</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
-        <v>11.2300001084805</v>
+        <v>8.292999863624569</v>
       </c>
       <c r="G49" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" t="n">
+        <v>2867</v>
+      </c>
+      <c r="I49" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="J49" t="n">
         <v>2</v>
       </c>
-      <c r="H49" t="n">
-        <v>10786</v>
-      </c>
-      <c r="I49" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>HNRNPU</t>
+          <t>HSPD1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2384,26 +2375,28 @@
         </is>
       </c>
       <c r="E50" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="F50" t="n">
+        <v>10.1199999451637</v>
+      </c>
+      <c r="G50" t="n">
         <v>2</v>
       </c>
-      <c r="F50" t="n">
-        <v>7.15200006961823</v>
-      </c>
-      <c r="G50" t="n">
-        <v>1</v>
-      </c>
       <c r="H50" t="n">
-        <v>26403</v>
+        <v>6179</v>
       </c>
       <c r="I50" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="J50" t="inlineStr"/>
+        <v>46.7</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>HSPB1</t>
+          <t>ILF3</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2422,28 +2415,25 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>6.53</v>
       </c>
       <c r="F51" t="n">
-        <v>8.292999863624569</v>
+        <v>16.6700005531311</v>
       </c>
       <c r="G51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H51" t="n">
-        <v>2867</v>
+        <v>39936</v>
       </c>
       <c r="I51" t="n">
-        <v>62.7</v>
-      </c>
-      <c r="J51" t="n">
-        <v>2</v>
+        <v>41</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>HSPD1</t>
+          <t>MFAP1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2458,23 +2448,23 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>4.16</v>
+        <v>2.04</v>
       </c>
       <c r="F52" t="n">
-        <v>10.1199999451637</v>
+        <v>15.0299996137619</v>
       </c>
       <c r="G52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H52" t="n">
-        <v>6179</v>
+        <v>16366</v>
       </c>
       <c r="I52" t="n">
-        <v>46.7</v>
+        <v>44.9</v>
       </c>
       <c r="J52" t="n">
         <v>1</v>
@@ -2483,7 +2473,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ILF3</t>
+          <t>MSN</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2498,30 +2488,29 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>6.53</v>
+        <v>5.17</v>
       </c>
       <c r="F53" t="n">
-        <v>16.6700005531311</v>
+        <v>21.8400001525879</v>
       </c>
       <c r="G53" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H53" t="n">
-        <v>39936</v>
+        <v>18584</v>
       </c>
       <c r="I53" t="n">
-        <v>41</v>
-      </c>
-      <c r="J53" t="inlineStr"/>
+        <v>46.1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MFAP1</t>
+          <t>MYH9</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2540,28 +2529,28 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>2.04</v>
+        <v>14.19</v>
       </c>
       <c r="F54" t="n">
-        <v>15.0299996137619</v>
+        <v>12.8600001335144</v>
       </c>
       <c r="G54" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H54" t="n">
-        <v>16366</v>
+        <v>66742</v>
       </c>
       <c r="I54" t="n">
-        <v>44.9</v>
+        <v>40.5</v>
       </c>
       <c r="J54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MSN</t>
+          <t>NCL</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2580,26 +2569,28 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>5.17</v>
+        <v>2.92</v>
       </c>
       <c r="F55" t="n">
-        <v>21.8400001525879</v>
+        <v>9.577000141143801</v>
       </c>
       <c r="G55" t="n">
         <v>2</v>
       </c>
       <c r="H55" t="n">
-        <v>18584</v>
+        <v>13021</v>
       </c>
       <c r="I55" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="J55" t="inlineStr"/>
+        <v>52</v>
+      </c>
+      <c r="J55" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MYH9</t>
+          <t>PABPC1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2618,28 +2609,25 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>14.19</v>
+        <v>4.77</v>
       </c>
       <c r="F56" t="n">
-        <v>12.8600001335144</v>
+        <v>9.905999898910521</v>
       </c>
       <c r="G56" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H56" t="n">
-        <v>66742</v>
+        <v>10968</v>
       </c>
       <c r="I56" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="J56" t="n">
-        <v>2</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>NCL</t>
+          <t>PCBP2</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2658,28 +2646,28 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>2.92</v>
+        <v>2.03</v>
       </c>
       <c r="F57" t="n">
-        <v>9.577000141143801</v>
+        <v>8.493000268936161</v>
       </c>
       <c r="G57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H57" t="n">
-        <v>13021</v>
+        <v>20288</v>
       </c>
       <c r="I57" t="n">
-        <v>52</v>
+        <v>45.3</v>
       </c>
       <c r="J57" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>PABPC1</t>
+          <t>PDIA3</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2698,26 +2686,28 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>4.77</v>
+        <v>2.52</v>
       </c>
       <c r="F58" t="n">
-        <v>9.905999898910521</v>
+        <v>10.4999996721745</v>
       </c>
       <c r="G58" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H58" t="n">
-        <v>10968</v>
+        <v>14255</v>
       </c>
       <c r="I58" t="n">
-        <v>43.3</v>
-      </c>
-      <c r="J58" t="inlineStr"/>
+        <v>44.9</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PCBP2</t>
+          <t>PDIA6</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2736,19 +2726,19 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>2.03</v>
+        <v>2.25</v>
       </c>
       <c r="F59" t="n">
-        <v>8.493000268936161</v>
+        <v>6.81800022721291</v>
       </c>
       <c r="G59" t="n">
         <v>1</v>
       </c>
       <c r="H59" t="n">
-        <v>20288</v>
+        <v>13479</v>
       </c>
       <c r="I59" t="n">
-        <v>45.3</v>
+        <v>45.6</v>
       </c>
       <c r="J59" t="n">
         <v>1</v>
@@ -2757,7 +2747,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PDIA3</t>
+          <t>PNN</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2776,19 +2766,19 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>2.52</v>
+        <v>2.01</v>
       </c>
       <c r="F60" t="n">
-        <v>10.4999996721745</v>
+        <v>7.94999971985817</v>
       </c>
       <c r="G60" t="n">
         <v>1</v>
       </c>
       <c r="H60" t="n">
-        <v>14255</v>
+        <v>50162</v>
       </c>
       <c r="I60" t="n">
-        <v>44.9</v>
+        <v>43.4</v>
       </c>
       <c r="J60" t="n">
         <v>1.5</v>
@@ -2797,7 +2787,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PDIA6</t>
+          <t>PUF60</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2812,23 +2802,23 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>2.25</v>
+        <v>6.65</v>
       </c>
       <c r="F61" t="n">
-        <v>6.81800022721291</v>
+        <v>15.3799995779991</v>
       </c>
       <c r="G61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H61" t="n">
-        <v>13479</v>
+        <v>63833</v>
       </c>
       <c r="I61" t="n">
-        <v>45.6</v>
+        <v>40.4</v>
       </c>
       <c r="J61" t="n">
         <v>1</v>
@@ -2837,7 +2827,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PNN</t>
+          <t>RPL10A</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2856,28 +2846,28 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>2.01</v>
+        <v>2.34</v>
       </c>
       <c r="F62" t="n">
-        <v>7.94999971985817</v>
+        <v>18.8899993896484</v>
       </c>
       <c r="G62" t="n">
         <v>1</v>
       </c>
       <c r="H62" t="n">
-        <v>50162</v>
+        <v>4434</v>
       </c>
       <c r="I62" t="n">
-        <v>43.4</v>
+        <v>47.2</v>
       </c>
       <c r="J62" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>PUF60</t>
+          <t>RPL14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2896,28 +2886,28 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>6.65</v>
+        <v>2</v>
       </c>
       <c r="F63" t="n">
-        <v>15.3799995779991</v>
+        <v>8.371999859809881</v>
       </c>
       <c r="G63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H63" t="n">
-        <v>63833</v>
+        <v>4486</v>
       </c>
       <c r="I63" t="n">
-        <v>40.4</v>
+        <v>50.1</v>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>RPL10A</t>
+          <t>RPL18</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2932,32 +2922,29 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>2.34</v>
+        <v>2.52</v>
       </c>
       <c r="F64" t="n">
-        <v>18.8899993896484</v>
+        <v>23.3999997377396</v>
       </c>
       <c r="G64" t="n">
         <v>1</v>
       </c>
       <c r="H64" t="n">
-        <v>4434</v>
+        <v>4672</v>
       </c>
       <c r="I64" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="J64" t="n">
-        <v>3.5</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>RPL13</t>
+          <t>RPL27A</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2976,28 +2963,28 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>1.67</v>
+        <v>2</v>
       </c>
       <c r="F65" t="n">
-        <v>15.1700004935265</v>
+        <v>7.43200033903122</v>
       </c>
       <c r="G65" t="n">
         <v>1</v>
       </c>
       <c r="H65" t="n">
-        <v>6912</v>
+        <v>5214</v>
       </c>
       <c r="I65" t="n">
-        <v>48.2</v>
+        <v>45.1</v>
       </c>
       <c r="J65" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>RPL14</t>
+          <t>RPL7</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3012,32 +2999,32 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>2</v>
+        <v>2.08</v>
       </c>
       <c r="F66" t="n">
-        <v>8.371999859809881</v>
+        <v>16.5299996733665</v>
       </c>
       <c r="G66" t="n">
         <v>1</v>
       </c>
       <c r="H66" t="n">
-        <v>4486</v>
+        <v>6981</v>
       </c>
       <c r="I66" t="n">
-        <v>50.1</v>
+        <v>46.3</v>
       </c>
       <c r="J66" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>RPL17</t>
+          <t>RPN1</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3056,19 +3043,19 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>1.8</v>
+        <v>2.23</v>
       </c>
       <c r="F67" t="n">
-        <v>14.6699994802475</v>
+        <v>3.95400002598763</v>
       </c>
       <c r="G67" t="n">
         <v>1</v>
       </c>
       <c r="H67" t="n">
-        <v>8348</v>
+        <v>11267</v>
       </c>
       <c r="I67" t="n">
-        <v>47</v>
+        <v>42.7</v>
       </c>
       <c r="J67" t="n">
         <v>1</v>
@@ -3077,7 +3064,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>RPL18</t>
+          <t>RPS15</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3096,26 +3083,25 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>2.52</v>
+        <v>2.07</v>
       </c>
       <c r="F68" t="n">
-        <v>23.3999997377396</v>
+        <v>12.4099999666214</v>
       </c>
       <c r="G68" t="n">
         <v>1</v>
       </c>
       <c r="H68" t="n">
-        <v>4672</v>
+        <v>5916</v>
       </c>
       <c r="I68" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="J68" t="inlineStr"/>
+        <v>45.8</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>RPL27A</t>
+          <t>RPS3A</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3134,28 +3120,28 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>2.38</v>
       </c>
       <c r="F69" t="n">
-        <v>7.43200033903122</v>
+        <v>15.1500001549721</v>
       </c>
       <c r="G69" t="n">
         <v>1</v>
       </c>
       <c r="H69" t="n">
-        <v>5214</v>
+        <v>7181</v>
       </c>
       <c r="I69" t="n">
-        <v>45.1</v>
+        <v>42.1</v>
       </c>
       <c r="J69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>RPL7</t>
+          <t>RPS8</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3170,23 +3156,23 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>2.08</v>
+        <v>2.76</v>
       </c>
       <c r="F70" t="n">
-        <v>16.5299996733665</v>
+        <v>10.5800002813339</v>
       </c>
       <c r="G70" t="n">
         <v>1</v>
       </c>
       <c r="H70" t="n">
-        <v>6981</v>
+        <v>5067</v>
       </c>
       <c r="I70" t="n">
-        <v>46.3</v>
+        <v>47.2</v>
       </c>
       <c r="J70" t="n">
         <v>1</v>
@@ -3195,7 +3181,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>RPL7A</t>
+          <t>RRBP1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3210,32 +3196,32 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>1.84</v>
+        <v>2</v>
       </c>
       <c r="F71" t="n">
-        <v>18.0500000715256</v>
+        <v>5.17700016498566</v>
       </c>
       <c r="G71" t="n">
         <v>1</v>
       </c>
       <c r="H71" t="n">
-        <v>9154</v>
+        <v>79242</v>
       </c>
       <c r="I71" t="n">
-        <v>42.4</v>
+        <v>44.4</v>
       </c>
       <c r="J71" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>RPN1</t>
+          <t>SEPTIN2</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3250,32 +3236,29 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>2.23</v>
+        <v>2</v>
       </c>
       <c r="F72" t="n">
-        <v>3.95400002598763</v>
+        <v>3.87800000607967</v>
       </c>
       <c r="G72" t="n">
         <v>1</v>
       </c>
       <c r="H72" t="n">
-        <v>11267</v>
+        <v>21905</v>
       </c>
       <c r="I72" t="n">
-        <v>42.7</v>
-      </c>
-      <c r="J72" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>RPS10P5</t>
+          <t>SERPINB9</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3294,26 +3277,25 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>1.86</v>
+        <v>2</v>
       </c>
       <c r="F73" t="n">
-        <v>8.523000031709669</v>
+        <v>2.65999995172024</v>
       </c>
       <c r="G73" t="n">
         <v>1</v>
       </c>
       <c r="H73" t="n">
-        <v>19412</v>
+        <v>4113</v>
       </c>
       <c r="I73" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="J73" t="inlineStr"/>
+        <v>53.4</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>RPS15</t>
+          <t>UBA52</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3328,30 +3310,32 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>2.07</v>
+        <v>2</v>
       </c>
       <c r="F74" t="n">
-        <v>12.4099999666214</v>
+        <v>10.1599998772144</v>
       </c>
       <c r="G74" t="n">
         <v>1</v>
       </c>
       <c r="H74" t="n">
-        <v>5916</v>
+        <v>2525</v>
       </c>
       <c r="I74" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="J74" t="inlineStr"/>
+        <v>53.2</v>
+      </c>
+      <c r="J74" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>RPS3A</t>
+          <t>YBX1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3366,82 +3350,76 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>2.38</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="F75" t="n">
-        <v>15.1500001549721</v>
+        <v>55.5599987506866</v>
       </c>
       <c r="G75" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H75" t="n">
-        <v>7181</v>
+        <v>19424</v>
       </c>
       <c r="I75" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="J75" t="n">
-        <v>1</v>
+        <v>44.7</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>RPS8</t>
+          <t>ADCY5</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>NonCandidate</t>
+          <t>T2DM_Control</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>RNA Pull-down</t>
+          <t>GWAS Literature</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>2.76</v>
+        <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>10.5800002813339</v>
+        <v>0</v>
       </c>
       <c r="G76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H76" t="n">
-        <v>5067</v>
+        <v>547773</v>
       </c>
       <c r="I76" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="J76" t="n">
-        <v>1</v>
+        <v>36.4</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>RRBP1</t>
+          <t>APPL1</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>NonCandidate</t>
+          <t>T2DM_Control</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>RNA Pull-down</t>
+          <t>GWAS Literature</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3450,114 +3428,118 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>5.17700016498566</v>
+        <v>0</v>
       </c>
       <c r="G77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H77" t="n">
-        <v>79242</v>
+        <v>37425</v>
       </c>
       <c r="I77" t="n">
-        <v>44.4</v>
+        <v>42.6</v>
       </c>
       <c r="J77" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SEPTIN2</t>
+          <t>ARAP1</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>NonCandidate</t>
+          <t>T2DM_Control</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>RNA Pull-down</t>
+          <t>GWAS Literature</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E78" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" t="n">
+        <v>122430</v>
+      </c>
+      <c r="I78" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="J78" t="n">
         <v>2</v>
       </c>
-      <c r="F78" t="n">
-        <v>3.87800000607967</v>
-      </c>
-      <c r="G78" t="n">
-        <v>1</v>
-      </c>
-      <c r="H78" t="n">
-        <v>21905</v>
-      </c>
-      <c r="I78" t="n">
-        <v>38</v>
-      </c>
-      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SERPINB9</t>
+          <t>CAMK1D</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>NonCandidate</t>
+          <t>T2DM_Control</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>RNA Pull-down</t>
+          <t>GWAS Literature</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>2.65999995172024</v>
+        <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H79" t="n">
-        <v>4113</v>
+        <v>48057</v>
       </c>
       <c r="I79" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="J79" t="inlineStr"/>
+        <v>38.1</v>
+      </c>
+      <c r="J79" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SERPINH1</t>
+          <t>CDKAL1</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>NonCandidate</t>
+          <t>T2DM_Control</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>RNA Pull-down</t>
+          <t>GWAS Literature</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3566,156 +3548,152 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>1.82</v>
+        <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>2.87100002169609</v>
+        <v>0</v>
       </c>
       <c r="G80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H80" t="n">
-        <v>11993</v>
+        <v>688950</v>
       </c>
       <c r="I80" t="n">
-        <v>63.3</v>
+        <v>38.6</v>
       </c>
       <c r="J80" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>TPM4</t>
+          <t>DGKB</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>NonCandidate</t>
+          <t>T2DM_Control</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>RNA Pull-down</t>
+          <t>GWAS Literature</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>1.66</v>
+        <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>6.0479998588562</v>
+        <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H81" t="n">
-        <v>15815</v>
+        <v>261485</v>
       </c>
       <c r="I81" t="n">
-        <v>42.6</v>
-      </c>
-      <c r="J81" t="n">
-        <v>1</v>
+        <v>36.4</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TUBB4B</t>
+          <t>DUSP8</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>NonCandidate</t>
+          <t>T2DM_Control</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>RNA Pull-down</t>
+          <t>GWAS Literature</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>1.54</v>
+        <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>10.5599999427795</v>
+        <v>0</v>
       </c>
       <c r="G82" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H82" t="n">
-        <v>4968</v>
+        <v>61280</v>
       </c>
       <c r="I82" t="n">
-        <v>50</v>
-      </c>
-      <c r="J82" t="inlineStr"/>
+        <v>36.1</v>
+      </c>
+      <c r="J82" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>UBA52</t>
+          <t>FOXA2</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>NonCandidate</t>
+          <t>T2DM_Control</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>RNA Pull-down</t>
+          <t>GWAS Literature</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>10.1599998772144</v>
+        <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H83" t="n">
-        <v>2525</v>
+        <v>3988</v>
       </c>
       <c r="I83" t="n">
-        <v>53.2</v>
-      </c>
-      <c r="J83" t="n">
-        <v>2</v>
+        <v>66.5</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>VAT1</t>
+          <t>FTO</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>NonCandidate</t>
+          <t>T2DM_Control</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>RNA Pull-down</t>
+          <t>GWAS Literature</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3724,66 +3702,68 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>1.43</v>
+        <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>6.87000006437302</v>
+        <v>0</v>
       </c>
       <c r="G84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H84" t="n">
-        <v>49551</v>
+        <v>220169</v>
       </c>
       <c r="I84" t="n">
-        <v>42.1</v>
+        <v>38.2</v>
       </c>
       <c r="J84" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>YBX1</t>
+          <t>GCK</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>NonCandidate</t>
+          <t>T2DM_Control</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>RNA Pull-down</t>
+          <t>GWAS Literature</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>8.279999999999999</v>
+        <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>55.5599987506866</v>
+        <v>0</v>
       </c>
       <c r="G85" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H85" t="n">
-        <v>19424</v>
+        <v>35461</v>
       </c>
       <c r="I85" t="n">
-        <v>44.7</v>
-      </c>
-      <c r="J85" t="inlineStr"/>
+        <v>60.9</v>
+      </c>
+      <c r="J85" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ADCY5</t>
+          <t>GCKR</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3811,17 +3791,19 @@
         <v>0</v>
       </c>
       <c r="H86" t="n">
-        <v>547773</v>
+        <v>27360</v>
       </c>
       <c r="I86" t="n">
-        <v>36.4</v>
-      </c>
-      <c r="J86" t="inlineStr"/>
+        <v>49.1</v>
+      </c>
+      <c r="J86" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>APPL1</t>
+          <t>GRB14</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3849,10 +3831,10 @@
         <v>0</v>
       </c>
       <c r="H87" t="n">
-        <v>37425</v>
+        <v>106288</v>
       </c>
       <c r="I87" t="n">
-        <v>42.6</v>
+        <v>42.2</v>
       </c>
       <c r="J87" t="n">
         <v>1</v>
@@ -3861,7 +3843,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ARAP1</t>
+          <t>HHEX</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -3889,19 +3871,19 @@
         <v>0</v>
       </c>
       <c r="H88" t="n">
-        <v>122430</v>
+        <v>27853</v>
       </c>
       <c r="I88" t="n">
-        <v>38.7</v>
+        <v>59.5</v>
       </c>
       <c r="J88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAMK1D</t>
+          <t>HMGA2</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3916,7 +3898,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -3929,19 +3911,16 @@
         <v>0</v>
       </c>
       <c r="H89" t="n">
-        <v>48057</v>
+        <v>77475</v>
       </c>
       <c r="I89" t="n">
-        <v>38.1</v>
-      </c>
-      <c r="J89" t="n">
-        <v>1.5</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CDKAL1</t>
+          <t>HNF1A</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3956,7 +3935,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -3969,19 +3948,16 @@
         <v>0</v>
       </c>
       <c r="H90" t="n">
-        <v>688950</v>
+        <v>31786</v>
       </c>
       <c r="I90" t="n">
-        <v>38.6</v>
-      </c>
-      <c r="J90" t="n">
-        <v>2.5</v>
+        <v>54.4</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>DGKB</t>
+          <t>HNF1B</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4009,17 +3985,16 @@
         <v>0</v>
       </c>
       <c r="H91" t="n">
-        <v>261485</v>
+        <v>59144</v>
       </c>
       <c r="I91" t="n">
-        <v>36.4</v>
-      </c>
-      <c r="J91" t="inlineStr"/>
+        <v>38.3</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>DUSP8</t>
+          <t>JAZF1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4047,19 +4022,19 @@
         <v>0</v>
       </c>
       <c r="H92" t="n">
-        <v>61280</v>
+        <v>290504</v>
       </c>
       <c r="I92" t="n">
-        <v>36.1</v>
+        <v>41.4</v>
       </c>
       <c r="J92" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>FOXA2</t>
+          <t>KCNJ11</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4074,7 +4049,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -4087,17 +4062,19 @@
         <v>0</v>
       </c>
       <c r="H93" t="n">
-        <v>3988</v>
+        <v>9625</v>
       </c>
       <c r="I93" t="n">
-        <v>66.5</v>
-      </c>
-      <c r="J93" t="inlineStr"/>
+        <v>46.2</v>
+      </c>
+      <c r="J93" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>FTO</t>
+          <t>KLF14</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4112,7 +4089,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -4125,19 +4102,19 @@
         <v>0</v>
       </c>
       <c r="H94" t="n">
-        <v>220169</v>
+        <v>8200</v>
       </c>
       <c r="I94" t="n">
-        <v>38.2</v>
+        <v>65</v>
       </c>
       <c r="J94" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>GCK</t>
+          <t>MNX1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4152,7 +4129,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -4165,19 +4142,16 @@
         <v>0</v>
       </c>
       <c r="H95" t="n">
-        <v>35461</v>
+        <v>7716</v>
       </c>
       <c r="I95" t="n">
-        <v>60.9</v>
-      </c>
-      <c r="J95" t="n">
-        <v>3</v>
+        <v>48.2</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>GCKR</t>
+          <t>PAM</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4192,7 +4166,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -4205,10 +4179,10 @@
         <v>0</v>
       </c>
       <c r="H96" t="n">
-        <v>27360</v>
+        <v>462588</v>
       </c>
       <c r="I96" t="n">
-        <v>49.1</v>
+        <v>36.6</v>
       </c>
       <c r="J96" t="n">
         <v>1</v>
@@ -4217,7 +4191,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>GRB14</t>
+          <t>PDX1</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4232,7 +4206,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E97" t="n">
@@ -4245,19 +4219,16 @@
         <v>0</v>
       </c>
       <c r="H97" t="n">
-        <v>106288</v>
+        <v>8856</v>
       </c>
       <c r="I97" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="J97" t="n">
-        <v>1</v>
+        <v>61.8</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>HHEX</t>
+          <t>PPARG</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4285,10 +4256,10 @@
         <v>0</v>
       </c>
       <c r="H98" t="n">
-        <v>27853</v>
+        <v>494639</v>
       </c>
       <c r="I98" t="n">
-        <v>59.5</v>
+        <v>38.7</v>
       </c>
       <c r="J98" t="n">
         <v>1</v>
@@ -4297,7 +4268,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>HMGA2</t>
+          <t>PROX1</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4325,17 +4296,19 @@
         <v>0</v>
       </c>
       <c r="H99" t="n">
-        <v>77475</v>
+        <v>49409</v>
       </c>
       <c r="I99" t="n">
-        <v>36.8</v>
-      </c>
-      <c r="J99" t="inlineStr"/>
+        <v>36.5</v>
+      </c>
+      <c r="J99" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>HNF1A</t>
+          <t>RREB1</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4350,7 +4323,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -4363,17 +4336,19 @@
         <v>0</v>
       </c>
       <c r="H100" t="n">
-        <v>31786</v>
+        <v>177238</v>
       </c>
       <c r="I100" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="J100" t="inlineStr"/>
+        <v>44</v>
+      </c>
+      <c r="J100" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>HNF1B</t>
+          <t>SLC16A11</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4388,7 +4363,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -4401,17 +4376,19 @@
         <v>0</v>
       </c>
       <c r="H101" t="n">
-        <v>59144</v>
+        <v>14520</v>
       </c>
       <c r="I101" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="J101" t="inlineStr"/>
+        <v>36.5</v>
+      </c>
+      <c r="J101" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>JAZF1</t>
+          <t>SLC30A8</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -4426,7 +4403,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -4439,19 +4416,16 @@
         <v>0</v>
       </c>
       <c r="H102" t="n">
-        <v>290504</v>
+        <v>110156</v>
       </c>
       <c r="I102" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="J102" t="n">
-        <v>2</v>
+        <v>40.2</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>KCNJ11</t>
+          <t>ST6GAL1</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4479,10 +4453,10 @@
         <v>0</v>
       </c>
       <c r="H103" t="n">
-        <v>9625</v>
+        <v>93218</v>
       </c>
       <c r="I103" t="n">
-        <v>46.2</v>
+        <v>37.7</v>
       </c>
       <c r="J103" t="n">
         <v>1.5</v>
@@ -4491,7 +4465,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>KLF14</t>
+          <t>TCF7L2</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -4519,19 +4493,16 @@
         <v>0</v>
       </c>
       <c r="H104" t="n">
-        <v>8200</v>
+        <v>224243</v>
       </c>
       <c r="I104" t="n">
-        <v>65</v>
-      </c>
-      <c r="J104" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>MNX1</t>
+          <t>TSPAN8</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4559,404 +4530,105 @@
         <v>0</v>
       </c>
       <c r="H105" t="n">
-        <v>7716</v>
+        <v>92696</v>
       </c>
       <c r="I105" t="n">
-        <v>48.2</v>
-      </c>
-      <c r="J105" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>PAM</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>T2DM_Control</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>GWAS Literature</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E106" t="n">
-        <v>0</v>
-      </c>
-      <c r="F106" t="n">
-        <v>0</v>
-      </c>
-      <c r="G106" t="n">
-        <v>0</v>
-      </c>
-      <c r="H106" t="n">
-        <v>462588</v>
-      </c>
-      <c r="I106" t="n">
-        <v>36.6</v>
-      </c>
-      <c r="J106" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>PDX1</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>T2DM_Control</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>GWAS Literature</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E107" t="n">
-        <v>0</v>
-      </c>
-      <c r="F107" t="n">
-        <v>0</v>
-      </c>
-      <c r="G107" t="n">
-        <v>0</v>
-      </c>
-      <c r="H107" t="n">
-        <v>8856</v>
-      </c>
-      <c r="I107" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="J107" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>PPARG</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>T2DM_Control</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>GWAS Literature</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E108" t="n">
-        <v>0</v>
-      </c>
-      <c r="F108" t="n">
-        <v>0</v>
-      </c>
-      <c r="G108" t="n">
-        <v>0</v>
-      </c>
-      <c r="H108" t="n">
-        <v>494639</v>
-      </c>
-      <c r="I108" t="n">
-        <v>38.7</v>
-      </c>
-      <c r="J108" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>PROX1</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>T2DM_Control</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>GWAS Literature</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E109" t="n">
-        <v>0</v>
-      </c>
-      <c r="F109" t="n">
-        <v>0</v>
-      </c>
-      <c r="G109" t="n">
-        <v>0</v>
-      </c>
-      <c r="H109" t="n">
-        <v>49409</v>
-      </c>
-      <c r="I109" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="J109" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>RREB1</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>T2DM_Control</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>GWAS Literature</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E110" t="n">
-        <v>0</v>
-      </c>
-      <c r="F110" t="n">
-        <v>0</v>
-      </c>
-      <c r="G110" t="n">
-        <v>0</v>
-      </c>
-      <c r="H110" t="n">
-        <v>177238</v>
-      </c>
-      <c r="I110" t="n">
-        <v>44</v>
-      </c>
-      <c r="J110" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>SLC16A11</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>T2DM_Control</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>GWAS Literature</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E111" t="n">
-        <v>0</v>
-      </c>
-      <c r="F111" t="n">
-        <v>0</v>
-      </c>
-      <c r="G111" t="n">
-        <v>0</v>
-      </c>
-      <c r="H111" t="n">
-        <v>14520</v>
-      </c>
-      <c r="I111" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="J111" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>SLC30A8</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>T2DM_Control</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>GWAS Literature</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E112" t="n">
-        <v>0</v>
-      </c>
-      <c r="F112" t="n">
-        <v>0</v>
-      </c>
-      <c r="G112" t="n">
-        <v>0</v>
-      </c>
-      <c r="H112" t="n">
-        <v>110156</v>
-      </c>
-      <c r="I112" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="J112" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>ST6GAL1</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>T2DM_Control</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>GWAS Literature</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E113" t="n">
-        <v>0</v>
-      </c>
-      <c r="F113" t="n">
-        <v>0</v>
-      </c>
-      <c r="G113" t="n">
-        <v>0</v>
-      </c>
-      <c r="H113" t="n">
-        <v>93218</v>
-      </c>
-      <c r="I113" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="J113" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>TCF7L2</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>T2DM_Control</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>GWAS Literature</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E114" t="n">
-        <v>0</v>
-      </c>
-      <c r="F114" t="n">
-        <v>0</v>
-      </c>
-      <c r="G114" t="n">
-        <v>0</v>
-      </c>
-      <c r="H114" t="n">
-        <v>224243</v>
-      </c>
-      <c r="I114" t="n">
-        <v>36</v>
-      </c>
-      <c r="J114" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>TSPAN8</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>T2DM_Control</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>GWAS Literature</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E115" t="n">
-        <v>0</v>
-      </c>
-      <c r="F115" t="n">
-        <v>0</v>
-      </c>
-      <c r="G115" t="n">
-        <v>0</v>
-      </c>
-      <c r="H115" t="n">
-        <v>92696</v>
-      </c>
-      <c r="I115" t="n">
         <v>42</v>
       </c>
-      <c r="J115" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>**Supplementary Table S1.** Gene list with group assignment, identification source, pull-down mass spectrometry metrics, and genomic covariates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>- **Gene:** HGNC gene symbol</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>- **Group:** Candidate (HOTAIR-binding protein), NonCandidate (HOTAIR-binding Unused≥2.0), T2DM_Control (T2DM GWAS literature genes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>- **Source:** RNA Pull-down (identified by mass spectrometry), Literature Curation (validated HOTAIR literature targets), GWAS Literature (known T2DM-associated genes from GWAS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>- **Analyzed:** Yes/No — whether the gene had eQTLGen weights available for S-PrediXcan analysis (19/30 candidates analyzed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>- **PD_Unused_Score:** Unused intensity score from RNA pull-down MS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>- **PD_Sequence_Coverage_Pct:** Sequence coverage percentage in pull-down MS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>- **PD_Peptides_95pct:** Number of peptides with ≥95% confidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>- **Gene_Length_bp:** Gene length in base pairs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>- **GC_Content_Pct:** GC content percentage</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>- **Mean_eQTL_SNP_Count:** Mean number of cis-eQTL SNPs across eQTLGen (where available)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>